<commit_message>
add description text files
</commit_message>
<xml_diff>
--- a/Part2/report_source/Part2_spreadsheet.xlsx
+++ b/Part2/report_source/Part2_spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chi-Han Chiu\Desktop\Viterbi_Decoder\instruction\Final Project\assignment itself\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F43FA6-77AC-4279-BAEE-BC37EEF2E81C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6424CDEB-9191-4CAA-B36D-5FFE2713A52B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -514,6 +514,9 @@
       <c r="H4">
         <v>256</v>
       </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -537,6 +540,9 @@
       <c r="H5">
         <v>256</v>
       </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -560,6 +566,9 @@
       <c r="H6">
         <v>256</v>
       </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -583,6 +592,9 @@
       <c r="H7">
         <v>256</v>
       </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -606,6 +618,9 @@
       <c r="H8">
         <v>256</v>
       </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -629,6 +644,9 @@
       <c r="H9">
         <v>232</v>
       </c>
+      <c r="I9">
+        <v>24</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -652,6 +670,9 @@
       <c r="H10">
         <v>243</v>
       </c>
+      <c r="I10">
+        <v>13</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -675,6 +696,9 @@
       <c r="H11">
         <v>238</v>
       </c>
+      <c r="I11">
+        <v>18</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -698,6 +722,9 @@
       <c r="H12">
         <v>253</v>
       </c>
+      <c r="I12">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -721,6 +748,9 @@
       <c r="H13">
         <v>256</v>
       </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -744,6 +774,9 @@
       <c r="H14">
         <v>249</v>
       </c>
+      <c r="I14">
+        <v>7</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -767,6 +800,9 @@
       <c r="H15">
         <v>250</v>
       </c>
+      <c r="I15">
+        <v>6</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -790,8 +826,11 @@
       <c r="H16">
         <v>254</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -813,8 +852,11 @@
       <c r="H17">
         <v>243</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I17">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -836,8 +878,11 @@
       <c r="H18">
         <v>251</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I18">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -858,6 +903,9 @@
       </c>
       <c r="H19">
         <v>250</v>
+      </c>
+      <c r="I19">
+        <v>6</v>
       </c>
     </row>
     <row r="1048441" spans="2:2" x14ac:dyDescent="0.25">

</xml_diff>